<commit_message>
fixed ghost row in register data
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PharmaConnectTestData.xlsx
+++ b/src/test/resources/testData/PharmaConnectTestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97F9A997-114C-41CB-8B1B-9B1646D2C916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{62403559-CEEF-4473-AFBB-936177CBB899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -852,7 +852,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E714C358-B9B9-4183-B981-A39021BBDAF9}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="2" customWidth="1"/>
@@ -1259,9 +1259,6 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="D15" s="1"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{5083AD58-E1AA-4851-BB0D-AF73B29FC447}"/>

</xml_diff>

<commit_message>
added new test data
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PharmaConnectTestData.xlsx
+++ b/src/test/resources/testData/PharmaConnectTestData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BD141A1-2D52-41B0-B280-1823CA88770C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{991907DF-1752-4389-8A2C-5067DCBD789C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="188">
   <si>
     <t>Test Name</t>
   </si>
@@ -486,24 +486,6 @@
   </si>
   <si>
     <t>Provide valid operating hours and verify it is accepted</t>
-  </si>
-  <si>
-    <t>Verify back to home navigation</t>
-  </si>
-  <si>
-    <t>Click back to home link and verify navigation to home page</t>
-  </si>
-  <si>
-    <t>/</t>
-  </si>
-  <si>
-    <t>Verify login page navigation</t>
-  </si>
-  <si>
-    <t>Click already registered login link and verify navigation to login page</t>
-  </si>
-  <si>
-    <t>/login</t>
   </si>
   <si>
     <t>FullName(*)</t>
@@ -651,7 +633,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -704,12 +686,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF3F3F3"/>
         <bgColor rgb="FFF3F3F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-        <bgColor rgb="FFFFE599"/>
       </patternFill>
     </fill>
   </fills>
@@ -778,7 +754,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -830,12 +806,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1445,7 +1415,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{940AA429-D4CB-410C-A8A6-132D3D9A19FE}">
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -2865,118 +2835,6 @@
       </c>
       <c r="R25" s="18" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18" ht="22.5">
-      <c r="A26" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="H26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="I26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="J26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="K26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="L26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="M26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="N26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="O26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="P26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q26" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="R26" s="18" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" ht="22.5">
-      <c r="A27" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="F27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="G27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="H27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="I27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="J27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="K27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="L27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="M27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="N27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="O27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="P27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q27" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="R27" s="20" t="s">
-        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3010,7 +2868,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D1" t="s">
         <v>49</v>
@@ -3022,7 +2880,7 @@
         <v>52</v>
       </c>
       <c r="G1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="H1" t="s">
         <v>53</v>
@@ -3031,21 +2889,21 @@
         <v>58</v>
       </c>
       <c r="J1" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="30.75">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D2" t="s">
         <v>66</v>
@@ -3065,13 +2923,13 @@
     </row>
     <row r="3" spans="1:11" ht="30.75">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
         <v>66</v>
@@ -3083,7 +2941,7 @@
         <v>125</v>
       </c>
       <c r="G3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="H3">
         <v>600001</v>
@@ -3100,16 +2958,16 @@
     </row>
     <row r="4" spans="1:11" ht="45.75">
       <c r="A4" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E4" t="s">
         <v>66</v>
@@ -3126,16 +2984,16 @@
     </row>
     <row r="5" spans="1:11" ht="80.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E5" t="s">
         <v>66</v>
@@ -3147,18 +3005,18 @@
         <v>10</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="60.75">
       <c r="A6" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>66</v>
@@ -3178,13 +3036,13 @@
     </row>
     <row r="7" spans="1:11" ht="60.75">
       <c r="A7" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C7" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>66</v>
@@ -3204,13 +3062,13 @@
     </row>
     <row r="8" spans="1:11" ht="60.75">
       <c r="A8" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>66</v>
@@ -3230,13 +3088,13 @@
     </row>
     <row r="9" spans="1:11" ht="45.75">
       <c r="A9" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>66</v>
@@ -3256,13 +3114,13 @@
     </row>
     <row r="10" spans="1:11" ht="45.75">
       <c r="A10" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>66</v>
@@ -3282,13 +3140,13 @@
     </row>
     <row r="11" spans="1:11" ht="45.75">
       <c r="A11" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C11" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>66</v>
@@ -3300,7 +3158,7 @@
         <v>12345678</v>
       </c>
       <c r="J11" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>144</v>
@@ -3308,13 +3166,13 @@
     </row>
     <row r="12" spans="1:11" ht="30.75">
       <c r="A12" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C12" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>66</v>
@@ -3337,13 +3195,13 @@
     </row>
     <row r="13" spans="1:11" ht="30.75">
       <c r="A13" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C13" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>66</v>
@@ -3366,13 +3224,13 @@
     </row>
     <row r="14" spans="1:11" ht="30.75">
       <c r="A14" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C14" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>66</v>

</xml_diff>